<commit_message>
GSE130613 - Fix step14_DE_only table: label unannotated genes, sort named genes first
</commit_message>
<xml_diff>
--- a/orthogonal_validation/results/tables/step14_spliced_only.xlsx
+++ b/orthogonal_validation/results/tables/step14_spliced_only.xlsx
@@ -17818,7 +17818,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>unannotated</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>unannotated</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">

</xml_diff>